<commit_message>
Read another workbook's cells from what the file cached of them
A formula such as [1]Sheet1!A1 or VLOOKUP(x,[1]Data!B:B,...) gave #REF!,
though the file keeps, under xl/externalLinks, the values Excel last read
from that workbook.  A sheet of a linked workbook is now a read-only model
of those values, read when a formula first asks for it, blank where the
link cached nothing.  It is no sheet of the workbook: it is not computed,
written or counted.  A link or sheet the file has not, and a sheet whose
refresh failed and cached nothing, are #REF!, and INDIRECT reaches none of
them, as Excel does with the other file closed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/links.xlsx
+++ b/test/fixtures/links.xlsx
@@ -12,6 +12,7 @@
   </externalReferences>
   <definedNames>
     <definedName name="othername">[1]!MonthNames</definedName>
+    <definedName name="named_cell">[1]Sheet1!$B$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
@@ -22,9 +23,47 @@
   <externalBook r:id="rId1">
     <sheetNames>
       <sheetName val="Sheet1"/>
+      <sheetName val="Gone"/>
+      <sheetName val="Empty"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="0">
+        <row r="1">
+          <cell r="A1">
+            <v>2</v>
+          </cell>
+          <cell r="B1">
+            <v>10</v>
+          </cell>
+          <cell r="C1" t="str">
+            <v>x</v>
+          </cell>
+          <cell r="D1" t="b">
+            <v>1</v>
+          </cell>
+          <cell r="E1" t="e">
+            <v>#N/A</v>
+          </cell>
+        </row>
+        <row r="2">
+          <cell r="A2">
+            <v>3</v>
+          </cell>
+          <cell r="B2">
+            <v>20</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="A3">
+            <v>4</v>
+          </cell>
+          <cell r="B3">
+            <v>30</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -32,24 +71,111 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B17"/>
   <sheetData>
     <row r="1">
       <c r="A1">
         <f>[1]Sheet1!$A$1</f>
         <v>2</v>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>SUM([1]Sheet1!$A$1:$B$2)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <f>SUM([1]Sheet1!A:A)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="e">
+        <f>[1]Nope!A1</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="e">
+        <f>INDIRECT("[1]Sheet1!A1")</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="e">
+        <f>[2]Sheet1!A1</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <f>VLOOKUP(3,[1]Sheet1!$A$1:$B$3,2,FALSE)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <f>[1]Sheet1!$D$1</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <f>[1]Sheet1!$C$1</f>
+        <v>x</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="e">
+        <f>[1]Sheet1!$E$1</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <f>[1]Sheet1!$F$1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <f>named_cell</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <f>SUM([1]Sheet1!$A$1:$C$5)</f>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <f>SHEETS()</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="e">
+        <f>[1]Gone!A1</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <f>[1]Empty!B7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
       <c r="B1" t="inlineStr">
         <is>
           <t>other.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Read the names of another workbook from what the file cached of them
[1]!Rate, [1]!'quoted name' and [1]Sheet1!Rate gave #ERROR! or #NAME?,
though the file keeps the names of the workbook it links to.  A name that
points at a range now reads the sheet of that workbook the file cached,
one that is #REF! there is #REF!, and one it has not is #NAME?.  A table
of that workbook and a DDE or OLE link are #REF!, as Excel caches them.
[0] names the workbook's own sheets and names.  INDIRECT still reaches no
name of another workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/links.xlsx
+++ b/test/fixtures/links.xlsx
@@ -9,6 +9,7 @@
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
+    <externalReference r:id="rId3"/>
   </externalReferences>
   <definedNames>
     <definedName name="othername">[1]!MonthNames</definedName>
@@ -26,6 +27,13 @@
       <sheetName val="Gone"/>
       <sheetName val="Empty"/>
     </sheetNames>
+    <definedNames>
+      <definedName name="Cell" refersTo="='Sheet1'!$A$1"/>
+      <definedName name="Range" refersTo="='Sheet1'!$A$1:$B$2"/>
+      <definedName name="Broken" refersTo="#REF!"/>
+      <definedName name="Local" refersTo="='Sheet1'!$B$3" sheetId="0"/>
+      <definedName name="Macro"/>
+    </definedNames>
     <sheetDataSet>
       <sheetData sheetId="0">
         <row r="1">
@@ -69,9 +77,19 @@
 </externalLink>
 </file>
 
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ddeLink ddeService="service" ddeTopic="topic">
+    <ddeItems>
+      <ddeItem name="Item" advise="1"/>
+    </ddeItems>
+  </ddeLink>
+</externalLink>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B26"/>
   <sheetData>
     <row r="1">
       <c r="A1">
@@ -105,7 +123,7 @@
     </row>
     <row r="6">
       <c r="A6" t="e">
-        <f>[2]Sheet1!A1</f>
+        <f>[7]Sheet1!A1</f>
         <v>#REF!</v>
       </c>
     </row>
@@ -116,13 +134,13 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8">
+      <c r="A8" t="b">
         <f>[1]Sheet1!$D$1</f>
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9">
+      <c r="A9" t="str">
         <f>[1]Sheet1!$C$1</f>
         <v>x</v>
       </c>
@@ -152,24 +170,78 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14">
-        <f>SHEETS()</f>
-        <v>1</v>
+      <c r="A14" t="e">
+        <f>[1]Gone!A1</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="e">
-        <f>[1]Gone!A1</f>
-        <v>#REF!</v>
+      <c r="A15">
+        <f>[1]Empty!B7</f>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <f>[1]Empty!B7</f>
-        <v>0</v>
+        <f>[1]!Cell</f>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
+      <c r="A17">
+        <f>SUM([1]!Range)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <f>[1]Sheet1!Local</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="e">
+        <f>[1]!Broken</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="e">
+        <f>[1]!Nope</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="e">
+        <f>[1]!Table1[c]</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="e">
+        <f>[2]!'Item'</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="e">
+        <f>INDIRECT("[1]!Cell")</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <f>[0]!named_cell</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="e">
+        <f>[1]!Macro</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="26">
       <c r="B1" t="inlineStr">
         <is>
           <t>other.xlsx</t>

</xml_diff>

<commit_message>
Keep a name that works out two references as written
umya read Sheet1!$H$5+Sheet1!$J$1 as one address, of the sheet
"Sheet1!$H$5+Sheet1", and wrote it back quoted so.  An address now
has at most one ! outside quotes and no operator; anything else is
kept whole, as {1,2;3,4} and IF(...) already were.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/links.xlsx
+++ b/test/fixtures/links.xlsx
@@ -14,6 +14,7 @@
   <definedNames>
     <definedName name="othername">[1]!MonthNames</definedName>
     <definedName name="named_cell">[1]Sheet1!$B$3</definedName>
+    <definedName name="pair">Sheet1!$A$1+Sheet1!$A$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
@@ -89,7 +90,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetData>
     <row r="1">
       <c r="A1">
@@ -242,6 +243,12 @@
       </c>
     </row>
     <row r="26">
+      <c r="A26">
+        <f>pair</f>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27">
       <c r="B1" t="inlineStr">
         <is>
           <t>other.xlsx</t>

</xml_diff>